<commit_message>
Reflect SEO consultant review into Excel management workbook
監修レビュー（鈴木謙一氏の公開発信ベース）の指摘を管理表に反映。

- 新規シート「⑥ 監修レビュー要点」：🔴🟠🟡の指摘と是正を一覧化
- ③ 3運用タイプ：PR TIMESの収益/KPIを「被リンク」→認知・指名検索・参照流入に是正
- ② キーワード戦略／各商品シート：量産ガードレール「1記事1オリジナル」を赤字注記
- ⑤ AI検索対策：llms.txtはGoogle非対応・過大評価しない旨を追記
- ① 概要：監修レビュー反映サマリーを追加

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UvmqjaSk6Q4EL44MiCWe3S
</commit_message>
<xml_diff>
--- a/suitcase-blog/libetee-suitcase-seo-plan.xlsx
+++ b/suitcase-blog/libetee-suitcase-seo-plan.xlsx
@@ -17,6 +17,7 @@
     <sheet name="留学アウトドアスーツケース" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="④ スケジュール" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="⑤ AI検索対策(LLMO)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="⑥ 監修レビュー要点" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +77,20 @@
     <font>
       <name val="Meiryo"/>
       <b val="1"/>
+      <color rgb="00B5462E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
       <color rgb="000F3B3A"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="001F2933"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -134,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -179,11 +192,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -715,217 +741,261 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="22" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>■ 監修レビュー反映（鈴木謙一氏の公開発信＝Google公式準拠のセルフチェック）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>PR TIMESは被リンク目的にしない：効果は認知・指名検索・参照流入で計測（→③運用タイプ）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>薄い量産をしない：1記事1オリジナル（一次情報を最低1つ）＝scaled content対策（→各商品シート注記）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>「第三者目線」は編集スタイル。実在著者＋実体験でE-E-A-T/Trustを担保。アフィリは独自の付加価値を必須。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>LLMOは過大評価しない：llms.txtはGoogle非対応。結局は質・信頼・構造化データ（→⑤AI検索対策）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>詳細は seo-strategy-review.md／⑥監修レビュー要点。施策前にGoogle検索セントラル・海外SEO情報ブログで一次確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
           <t>■ 進捗ダッシュボード（各商品シートから自動集計）</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>商品シート</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>計画記事数</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>公開済み</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>執筆中</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>公開率</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>PCスーツケース</t>
         </is>
       </c>
-      <c r="B31" s="7">
+      <c r="B38" s="7">
         <f>COUNTA('PCスーツケース'!$B$5:$B$60)</f>
         <v/>
       </c>
-      <c r="C31" s="7">
+      <c r="C38" s="7">
         <f>COUNTIF('PCスーツケース'!$N$5:$N$60,"公開済み")</f>
         <v/>
       </c>
-      <c r="D31" s="7">
+      <c r="D38" s="7">
         <f>COUNTIF('PCスーツケース'!$N$5:$N$60,"執筆中")</f>
         <v/>
       </c>
-      <c r="E31" s="7">
+      <c r="E38" s="7">
         <f>COUNTIF('PCスーツケース'!$N$5:$N$60,"未着手")</f>
         <v/>
       </c>
-      <c r="F31" s="8">
-        <f>IFERROR(C31/B31,0)</f>
+      <c r="F38" s="8">
+        <f>IFERROR(C38/B38,0)</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>クラシックアルミニウムスーツケース</t>
         </is>
       </c>
-      <c r="B32" s="7">
+      <c r="B39" s="7">
         <f>COUNTA('クラシックアルミニウムスーツケース'!$B$5:$B$60)</f>
         <v/>
       </c>
-      <c r="C32" s="7">
+      <c r="C39" s="7">
         <f>COUNTIF('クラシックアルミニウムスーツケース'!$N$5:$N$60,"公開済み")</f>
         <v/>
       </c>
-      <c r="D32" s="7">
+      <c r="D39" s="7">
         <f>COUNTIF('クラシックアルミニウムスーツケース'!$N$5:$N$60,"執筆中")</f>
         <v/>
       </c>
-      <c r="E32" s="7">
+      <c r="E39" s="7">
         <f>COUNTIF('クラシックアルミニウムスーツケース'!$N$5:$N$60,"未着手")</f>
         <v/>
       </c>
-      <c r="F32" s="8">
-        <f>IFERROR(C32/B32,0)</f>
+      <c r="F39" s="8">
+        <f>IFERROR(C39/B39,0)</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>多機能アルミニウムスーツケース</t>
         </is>
       </c>
-      <c r="B33" s="7">
+      <c r="B40" s="7">
         <f>COUNTA('多機能アルミニウムスーツケース'!$B$5:$B$60)</f>
         <v/>
       </c>
-      <c r="C33" s="7">
+      <c r="C40" s="7">
         <f>COUNTIF('多機能アルミニウムスーツケース'!$N$5:$N$60,"公開済み")</f>
         <v/>
       </c>
-      <c r="D33" s="7">
+      <c r="D40" s="7">
         <f>COUNTIF('多機能アルミニウムスーツケース'!$N$5:$N$60,"執筆中")</f>
         <v/>
       </c>
-      <c r="E33" s="7">
+      <c r="E40" s="7">
         <f>COUNTIF('多機能アルミニウムスーツケース'!$N$5:$N$60,"未着手")</f>
         <v/>
       </c>
-      <c r="F33" s="8">
-        <f>IFERROR(C33/B33,0)</f>
+      <c r="F40" s="8">
+        <f>IFERROR(C40/B40,0)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>ジップタイプスーツケース</t>
         </is>
       </c>
-      <c r="B34" s="7">
+      <c r="B41" s="7">
         <f>COUNTA('ジップタイプスーツケース'!$B$5:$B$60)</f>
         <v/>
       </c>
-      <c r="C34" s="7">
+      <c r="C41" s="7">
         <f>COUNTIF('ジップタイプスーツケース'!$N$5:$N$60,"公開済み")</f>
         <v/>
       </c>
-      <c r="D34" s="7">
+      <c r="D41" s="7">
         <f>COUNTIF('ジップタイプスーツケース'!$N$5:$N$60,"執筆中")</f>
         <v/>
       </c>
-      <c r="E34" s="7">
+      <c r="E41" s="7">
         <f>COUNTIF('ジップタイプスーツケース'!$N$5:$N$60,"未着手")</f>
         <v/>
       </c>
-      <c r="F34" s="8">
-        <f>IFERROR(C34/B34,0)</f>
+      <c r="F41" s="8">
+        <f>IFERROR(C41/B41,0)</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>留学アウトドアスーツケース</t>
         </is>
       </c>
-      <c r="B35" s="7">
+      <c r="B42" s="7">
         <f>COUNTA('留学アウトドアスーツケース'!$B$5:$B$60)</f>
         <v/>
       </c>
-      <c r="C35" s="7">
+      <c r="C42" s="7">
         <f>COUNTIF('留学アウトドアスーツケース'!$N$5:$N$60,"公開済み")</f>
         <v/>
       </c>
-      <c r="D35" s="7">
+      <c r="D42" s="7">
         <f>COUNTIF('留学アウトドアスーツケース'!$N$5:$N$60,"執筆中")</f>
         <v/>
       </c>
-      <c r="E35" s="7">
+      <c r="E42" s="7">
         <f>COUNTIF('留学アウトドアスーツケース'!$N$5:$N$60,"未着手")</f>
         <v/>
       </c>
-      <c r="F35" s="8">
-        <f>IFERROR(C35/B35,0)</f>
+      <c r="F42" s="8">
+        <f>IFERROR(C42/B42,0)</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B36" s="10">
-        <f>SUM(B31:B35)</f>
+      <c r="B43" s="10">
+        <f>SUM(B38:B42)</f>
         <v/>
       </c>
-      <c r="C36" s="10">
-        <f>SUM(C31:C35)</f>
+      <c r="C43" s="10">
+        <f>SUM(C38:C42)</f>
         <v/>
       </c>
-      <c r="D36" s="10">
-        <f>SUM(D31:D35)</f>
+      <c r="D43" s="10">
+        <f>SUM(D38:D42)</f>
         <v/>
       </c>
-      <c r="E36" s="10">
-        <f>SUM(E31:E35)</f>
+      <c r="E43" s="10">
+        <f>SUM(E38:E42)</f>
         <v/>
       </c>
-      <c r="F36" s="11">
-        <f>IFERROR(C36/B36,0)</f>
+      <c r="F43" s="11">
+        <f>IFERROR(C43/B43,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="29">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A4:F4"/>
@@ -934,9 +1004,13 @@
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:F7"/>
@@ -973,7 +1047,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>生成AIは「引用しやすい一次情報・明快な構造・第三者言及」を好む。SEOと両輪で仕込む。</t>
+          <t>生成AIは「引用しやすい一次情報・明快な構造・第三者言及」を好む。※特別な裏技はなく、結局は質・信頼・構造化が効く（監修レビュー反映）。過大評価しない。</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1278,7 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>llms.txt / 明快なsite構造</t>
+          <t>明快なsite構造（llms.txtは任意）</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
@@ -1214,7 +1288,7 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>主要ページ要約のllms.txt設置・内部リンク整理</t>
+          <t>内部リンク整理・要約文設置。※llms.txtはGoogle非対応、過度に期待しない</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -1237,6 +1311,250 @@
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>監修レビュー要点｜Google公式準拠のブラッシュアップ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SEO専門家・鈴木謙一氏の公開発信（海外SEO情報ブログ＋Google検索セントラル）に基づくセルフチェック。※本人監修ではありません。🔴＝公開前の必須修正。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>優先</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>指摘</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>なぜ（Google公式の考え方）</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>このプランでの是正</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>PR TIMESの被リンクでSEOは上がらない</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>配信リンクはnofollow/sponsored相当。順位目的の大量リンクはスパム扱いのリスク</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>③運用タイプのPR TIMES欄を「認知・指名検索・参照流入」に是正。KPIから被リンクを除外</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>掛け合わせKWの量産は低品質リスク</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>scaled content abuse／helpful contentの観点で薄い量産はサイト評価を下げる</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>②と各商品シートに「1記事1オリジナル(一次情報必須)」を注記</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>ペルソナで第三者を装うのは危険</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>レビュー評価とTrustは実使用の一次体験を重視。ステマ規制にも抵触</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>「第三者目線」は編集スタイルに限定。実在著者＋実体験を必須化</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>E-E-A-T（特にTrust/Experience）の作り込み</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>作り手の身元・一次体験が信頼につながる</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>運営者/著者/保証ページ整備。ボーケン試験=一次情報として前面(強み)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>アフィリ/比較は独自の付加価値が前提</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>寄せ集め比較は評価されない。独自の計測・視点・実使用が必要</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>比較表に独自列(実測重量/静音性の体感等)。理由つきで推奨を明言</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>キーワード起点→検索意図/トピック起点</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>単体ビッグワードは無理に狙わず、意図を満たす網羅で面を取る</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>②を検索意図ベースに。カニバリ対策(PC=ジップ)は対応済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>LLMO/AI検索を過大評価しない</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>AI検索でも効くのは質・信頼・構造化。llms.txtはGoogle非対応</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>⑤の重心を構造化データ・E-E-A-T・一次情報へ。llms.txtは任意扱い</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>技術SEOの明記</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>構造化データ・Core Web Vitals・モバイルはページ体験の前提</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Product/FAQ/Breadcrumb・表示速度・モバイル可読性を実装項目に</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>※ ポリシー名・時期は変わりうる。施策決定前にGoogle検索セントラルと海外SEO情報ブログの最新記事で必ず一次確認（＝本レビューの根本精神：公式に忠実に）。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1248,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1744,10 +2062,18 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>🔴監修レビュー反映：掛け合わせKWの数だけ薄い記事を量産しない。1記事1オリジナル(一次情報必須)。検索意図が同じ記事はまとめる(カニバリ回避)。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A17:H17"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1802,7 +2128,7 @@
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>狙い</t>
         </is>
@@ -1824,7 +2150,7 @@
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>媒体</t>
         </is>
@@ -1846,7 +2172,7 @@
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>目線・トーン</t>
         </is>
@@ -1868,7 +2194,7 @@
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>主担当</t>
         </is>
@@ -1890,7 +2216,7 @@
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>広告</t>
         </is>
@@ -1912,7 +2238,7 @@
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>CTA・リンク先</t>
         </is>
@@ -1934,7 +2260,7 @@
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>収益</t>
         </is>
@@ -1951,12 +2277,12 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>（間接）指名検索・被リンクでSEO底上げ</t>
+          <t>（間接）認知・指名検索・参照流入 ※被リンク効果は期待しない</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
@@ -1973,12 +2299,12 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>掲載数・被リンク数・参照流入</t>
+          <t>掲載数・参照流入・指名検索数 ※被リンクは指標にしない</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>コンプラ注意</t>
         </is>
@@ -2014,7 +2340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2176,8 +2502,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M5" s="17" t="inlineStr"/>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr"/>
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2240,8 +2566,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M6" s="17" t="inlineStr"/>
-      <c r="N6" s="17" t="inlineStr">
+      <c r="M6" s="18" t="inlineStr"/>
+      <c r="N6" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2304,8 +2630,8 @@
           <t>比較ページ(自社+他社)</t>
         </is>
       </c>
-      <c r="M7" s="17" t="inlineStr"/>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="M7" s="18" t="inlineStr"/>
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2368,8 +2694,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M8" s="17" t="inlineStr"/>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="M8" s="18" t="inlineStr"/>
+      <c r="N8" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2432,8 +2758,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr"/>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="M9" s="18" t="inlineStr"/>
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2496,8 +2822,8 @@
           <t>自社ブログ→EC</t>
         </is>
       </c>
-      <c r="M10" s="17" t="inlineStr"/>
-      <c r="N10" s="17" t="inlineStr">
+      <c r="M10" s="18" t="inlineStr"/>
+      <c r="N10" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2510,9 +2836,17 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>🔴監修レビュー反映：各記事は「1記事1オリジナル」。実測・実使用・ボーケン試験等の一次情報を最低1つ必ず入れる（検索意図が同じ薄い記事の量産はしない＝scaled content対策）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -2543,7 +2877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2705,8 +3039,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M5" s="17" t="inlineStr"/>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr"/>
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2769,8 +3103,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M6" s="17" t="inlineStr"/>
-      <c r="N6" s="17" t="inlineStr">
+      <c r="M6" s="18" t="inlineStr"/>
+      <c r="N6" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2833,8 +3167,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M7" s="17" t="inlineStr"/>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="M7" s="18" t="inlineStr"/>
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2897,8 +3231,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M8" s="17" t="inlineStr"/>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="M8" s="18" t="inlineStr"/>
+      <c r="N8" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -2961,8 +3295,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr"/>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="M9" s="18" t="inlineStr"/>
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3025,8 +3359,8 @@
           <t>自社ブログ→EC</t>
         </is>
       </c>
-      <c r="M10" s="17" t="inlineStr"/>
-      <c r="N10" s="17" t="inlineStr">
+      <c r="M10" s="18" t="inlineStr"/>
+      <c r="N10" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3039,9 +3373,17 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>🔴監修レビュー反映：各記事は「1記事1オリジナル」。実測・実使用・ボーケン試験等の一次情報を最低1つ必ず入れる（検索意図が同じ薄い記事の量産はしない＝scaled content対策）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3072,7 +3414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3234,8 +3576,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M5" s="17" t="inlineStr"/>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr"/>
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3298,8 +3640,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M6" s="17" t="inlineStr"/>
-      <c r="N6" s="17" t="inlineStr">
+      <c r="M6" s="18" t="inlineStr"/>
+      <c r="N6" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3362,8 +3704,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M7" s="17" t="inlineStr"/>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="M7" s="18" t="inlineStr"/>
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3426,8 +3768,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M8" s="17" t="inlineStr"/>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="M8" s="18" t="inlineStr"/>
+      <c r="N8" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3490,8 +3832,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr"/>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="M9" s="18" t="inlineStr"/>
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3554,8 +3896,8 @@
           <t>自社ブログ→EC</t>
         </is>
       </c>
-      <c r="M10" s="17" t="inlineStr"/>
-      <c r="N10" s="17" t="inlineStr">
+      <c r="M10" s="18" t="inlineStr"/>
+      <c r="N10" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3568,9 +3910,17 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>🔴監修レビュー反映：各記事は「1記事1オリジナル」。実測・実使用・ボーケン試験等の一次情報を最低1つ必ず入れる（検索意図が同じ薄い記事の量産はしない＝scaled content対策）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3601,7 +3951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3763,8 +4113,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M5" s="17" t="inlineStr"/>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr"/>
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3827,8 +4177,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M6" s="17" t="inlineStr"/>
-      <c r="N6" s="17" t="inlineStr">
+      <c r="M6" s="18" t="inlineStr"/>
+      <c r="N6" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3891,8 +4241,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M7" s="17" t="inlineStr"/>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="M7" s="18" t="inlineStr"/>
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -3955,8 +4305,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M8" s="17" t="inlineStr"/>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="M8" s="18" t="inlineStr"/>
+      <c r="N8" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4019,8 +4369,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr"/>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="M9" s="18" t="inlineStr"/>
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4083,8 +4433,8 @@
           <t>自社ブログ→EC</t>
         </is>
       </c>
-      <c r="M10" s="17" t="inlineStr"/>
-      <c r="N10" s="17" t="inlineStr">
+      <c r="M10" s="18" t="inlineStr"/>
+      <c r="N10" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4097,9 +4447,17 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>🔴監修レビュー反映：各記事は「1記事1オリジナル」。実測・実使用・ボーケン試験等の一次情報を最低1つ必ず入れる（検索意図が同じ薄い記事の量産はしない＝scaled content対策）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -4130,7 +4488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4292,8 +4650,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M5" s="17" t="inlineStr"/>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr"/>
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4356,8 +4714,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M6" s="17" t="inlineStr"/>
-      <c r="N6" s="17" t="inlineStr">
+      <c r="M6" s="18" t="inlineStr"/>
+      <c r="N6" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4420,8 +4778,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M7" s="17" t="inlineStr"/>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="M7" s="18" t="inlineStr"/>
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4484,8 +4842,8 @@
           <t>比較ページ</t>
         </is>
       </c>
-      <c r="M8" s="17" t="inlineStr"/>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="M8" s="18" t="inlineStr"/>
+      <c r="N8" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4548,8 +4906,8 @@
           <t>自社EC 商品ページ</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr"/>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="M9" s="18" t="inlineStr"/>
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4612,8 +4970,8 @@
           <t>自社ブログ→EC</t>
         </is>
       </c>
-      <c r="M10" s="17" t="inlineStr"/>
-      <c r="N10" s="17" t="inlineStr">
+      <c r="M10" s="18" t="inlineStr"/>
+      <c r="N10" s="18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4626,9 +4984,17 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>🔴監修レビュー反映：各記事は「1記事1オリジナル」。実測・実使用・ボーケン試験等の一次情報を最低1つ必ず入れる（検索意図が同じ薄い記事の量産はしない＝scaled content対策）。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>